<commit_message>
Refresh 2026-2027 fee and ledger data
Updated the source fee, invoice, and stock Excel files and regenerated the derived JSON datasets. This includes corrected textbook amounts across primary classes and the corresponding student balances, outstanding totals, and generated metadata timestamps. The changes reflect the latest 2026-2027 fee sheet and invoice outputs.
</commit_message>
<xml_diff>
--- a/source/INVOICE.xlsx
+++ b/source/INVOICE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A416FF2D-AB63-4108-986C-8558ABD615E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75505F5C-EDCB-4D0D-BB41-EDB85E88C68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -876,7 +876,7 @@
         <v>5000</v>
       </c>
       <c r="H7" s="8">
-        <v>25550</v>
+        <v>25490</v>
       </c>
       <c r="I7" s="10">
         <v>11330</v>
@@ -904,7 +904,7 @@
       </c>
       <c r="Q7" s="17">
         <f t="shared" si="0"/>
-        <v>115380</v>
+        <v>115320</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -930,7 +930,7 @@
         <v>5000</v>
       </c>
       <c r="H8" s="8">
-        <v>25730</v>
+        <v>25670</v>
       </c>
       <c r="I8" s="10">
         <v>11330</v>
@@ -958,7 +958,7 @@
       </c>
       <c r="Q8" s="17">
         <f t="shared" si="0"/>
-        <v>115560</v>
+        <v>115500</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>5000</v>
       </c>
       <c r="H9" s="8">
-        <v>26890</v>
+        <v>26830</v>
       </c>
       <c r="I9" s="10">
         <v>13230</v>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="Q9" s="17">
         <f t="shared" si="0"/>
-        <v>118620</v>
+        <v>118560</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1038,7 +1038,7 @@
         <v>5000</v>
       </c>
       <c r="H10" s="8">
-        <v>26910</v>
+        <v>26850</v>
       </c>
       <c r="I10" s="10">
         <v>13230</v>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="Q10" s="17">
         <f t="shared" si="0"/>
-        <v>118640</v>
+        <v>118580</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
@@ -1092,7 +1092,7 @@
         <v>5000</v>
       </c>
       <c r="H11" s="8">
-        <v>28850</v>
+        <v>28790</v>
       </c>
       <c r="I11" s="10">
         <v>13230</v>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="Q11" s="17">
         <f t="shared" si="0"/>
-        <v>120580</v>
+        <v>120520</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>